<commit_message>
Job 1 output: test prescribed period fixes (708→A, 729→B, 757→E, 810→A)
- 365/367 sections placed, 0 teacher conflicts, 0 room double-bookings
- All 4 prescribed periods honored correctly
- 0 consecutive-6 violations, 0 load violations
- 2 unplaced: 570 (McConnell), 710 (Saggio) — same as prior run

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Preflight_Validation_Report.xlsx
+++ b/Preflight_Validation_Report.xlsx
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>0</v>
+        <v>126</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
@@ -652,7 +652,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>961</v>
+        <v>1087</v>
       </c>
       <c r="C12" s="5" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Job 1 output: 366/366 placed after removing 723, 741 Psych #1 now placed
All sections placed with zero unplaced. Saggio's 741 Psychology sec#1
placed in Period D S1 after removing 723 Intro to Political Science
(8 enrollments) freed S2 capacity.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Preflight_Validation_Report.xlsx
+++ b/Preflight_Validation_Report.xlsx
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
@@ -652,7 +652,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>1087</v>
+        <v>1094</v>
       </c>
       <c r="C12" s="5" t="inlineStr"/>
     </row>
@@ -1263,7 +1263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1338,21 +1338,21 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="n">
-        <v>113184</v>
+        <v>114903</v>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Bardales, Carlos</t>
+          <t>Aslanyan, Nicholas</t>
         </is>
       </c>
       <c r="C2" s="5" t="n">
         <v>10</v>
       </c>
       <c r="D2" s="10" t="n">
-        <v>32.5</v>
+        <v>27.5</v>
       </c>
       <c r="E2" s="11" t="n">
-        <v>2.5</v>
+        <v>7.5</v>
       </c>
       <c r="F2" s="10" t="n">
         <v>6.5</v>
@@ -1365,23 +1365,23 @@
       </c>
       <c r="I2" s="12" t="inlineStr">
         <is>
-          <t>All core present — missing elective</t>
+          <t>Language</t>
         </is>
       </c>
       <c r="J2" s="13" t="inlineStr">
         <is>
-          <t>120 American Literature (English, 5.0cr, 1.0slot); 320 Spanish II (Language, 5.0cr, 1.0slot); 420 Geometry (Mathematics, 5.0cr, 1.0slot); 520 Chemistry (Science, 5.0cr, 1.0slot); 620 Driver's Ed/PE (Physical Education, 2.5cr, 0.5slot); 720 U.S. History I (Social Studies, 5.0cr, 1.0slot); 820 Theology 10 (Theology, 5.0cr, 1.0slot)</t>
+          <t>122 American Literature (English, 5.0cr, 1.0slot); 422 Geometry (Mathematics, 5.0cr, 1.0slot); 510 Biology (Science, 5.0cr, 1.0slot); 620 Driver's Ed/PE (Physical Education, 2.5cr, 0.5slot); 720 U.S. History I (Social Studies, 5.0cr, 1.0slot); 820 Theology 10 (Theology, 5.0cr, 1.0slot); 955 Academic Support (Special Education, 0.0cr, 1.0slot [0cr, 1 slot])</t>
         </is>
       </c>
       <c r="K2" s="9" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
-        <v>121287</v>
+        <v>113184</v>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Elliott, Michael</t>
+          <t>Bardales, Carlos</t>
         </is>
       </c>
       <c r="C3" s="5" t="n">
@@ -1409,18 +1409,18 @@
       </c>
       <c r="J3" s="13" t="inlineStr">
         <is>
-          <t>122 American Literature (English, 5.0cr, 1.0slot); 320 Spanish II (Language, 5.0cr, 1.0slot); 422 Geometry (Mathematics, 5.0cr, 1.0slot); 520 Chemistry (Science, 5.0cr, 1.0slot); 620 Driver's Ed/PE (Physical Education, 2.5cr, 0.5slot); 720 U.S. History I (Social Studies, 5.0cr, 1.0slot); 820 Theology 10 (Theology, 5.0cr, 1.0slot)</t>
+          <t>120 American Literature (English, 5.0cr, 1.0slot); 320 Spanish II (Language, 5.0cr, 1.0slot); 420 Geometry (Mathematics, 5.0cr, 1.0slot); 520 Chemistry (Science, 5.0cr, 1.0slot); 620 Driver's Ed/PE (Physical Education, 2.5cr, 0.5slot); 720 U.S. History I (Social Studies, 5.0cr, 1.0slot); 820 Theology 10 (Theology, 5.0cr, 1.0slot)</t>
         </is>
       </c>
       <c r="K3" s="9" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
-        <v>117427</v>
+        <v>113047</v>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Irving, Corey</t>
+          <t>Chittoni, Mario Enrico</t>
         </is>
       </c>
       <c r="C4" s="5" t="n">
@@ -1448,18 +1448,18 @@
       </c>
       <c r="J4" s="13" t="inlineStr">
         <is>
-          <t>120 American Literature (English, 5.0cr, 1.0slot); 315 Latin I H (Language, 5.0cr, 1.0slot); 420 Geometry (Mathematics, 5.0cr, 1.0slot); 520 Chemistry (Science, 5.0cr, 1.0slot); 620 Driver's Ed/PE (Physical Education, 2.5cr, 0.5slot); 711 World History H (Social Studies, 5.0cr, 1.0slot); 820 Theology 10 (Theology, 5.0cr, 1.0slot)</t>
+          <t>121 American Literature H (English, 5.0cr, 1.0slot); 327 Latin II H (Language, 5.0cr, 1.0slot); 420 Geometry (Mathematics, 5.0cr, 1.0slot); 521 Chemistry H (Science, 5.0cr, 1.0slot); 620 Driver's Ed/PE (Physical Education, 2.5cr, 0.5slot); 721 U.S. History I H (Social Studies, 5.0cr, 1.0slot); 820 Theology 10 (Theology, 5.0cr, 1.0slot)</t>
         </is>
       </c>
       <c r="K4" s="9" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>109385</v>
+        <v>121287</v>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Saliba, Georges</t>
+          <t>Elliott, Michael</t>
         </is>
       </c>
       <c r="C5" s="5" t="n">
@@ -1482,23 +1482,23 @@
       </c>
       <c r="I5" s="12" t="inlineStr">
         <is>
-          <t>Physical Education</t>
+          <t>All core present — missing elective</t>
         </is>
       </c>
       <c r="J5" s="13" t="inlineStr">
         <is>
-          <t>120 American Literature (English, 5.0cr, 1.0slot); 327 Latin II H (Language, 5.0cr, 1.0slot); 420 Geometry (Mathematics, 5.0cr, 1.0slot); 520 Chemistry (Science, 5.0cr, 1.0slot); 580 Robotics Engineering (Engineering, 2.5cr, 0.5slot); 720 U.S. History I (Social Studies, 5.0cr, 1.0slot); 820 Theology 10 (Theology, 5.0cr, 1.0slot)</t>
+          <t>122 American Literature (English, 5.0cr, 1.0slot); 320 Spanish II (Language, 5.0cr, 1.0slot); 422 Geometry (Mathematics, 5.0cr, 1.0slot); 520 Chemistry (Science, 5.0cr, 1.0slot); 620 Driver's Ed/PE (Physical Education, 2.5cr, 0.5slot); 720 U.S. History I (Social Studies, 5.0cr, 1.0slot); 820 Theology 10 (Theology, 5.0cr, 1.0slot)</t>
         </is>
       </c>
       <c r="K5" s="9" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>113831</v>
+        <v>117427</v>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Sanchez, Cordero</t>
+          <t>Irving, Corey</t>
         </is>
       </c>
       <c r="C6" s="5" t="n">
@@ -1526,22 +1526,22 @@
       </c>
       <c r="J6" s="13" t="inlineStr">
         <is>
-          <t>120 American Literature (English, 5.0cr, 1.0slot); 321 Spanish II H (Language, 5.0cr, 1.0slot); 421 Geometry H (Mathematics, 5.0cr, 1.0slot); 520 Chemistry (Science, 5.0cr, 1.0slot); 620 Driver's Ed/PE (Physical Education, 2.5cr, 0.5slot); 721 U.S. History I H (Social Studies, 5.0cr, 1.0slot); 820 Theology 10 (Theology, 5.0cr, 1.0slot)</t>
+          <t>120 American Literature (English, 5.0cr, 1.0slot); 315 Latin I H (Language, 5.0cr, 1.0slot); 420 Geometry (Mathematics, 5.0cr, 1.0slot); 520 Chemistry (Science, 5.0cr, 1.0slot); 620 Driver's Ed/PE (Physical Education, 2.5cr, 0.5slot); 711 World History H (Social Studies, 5.0cr, 1.0slot); 820 Theology 10 (Theology, 5.0cr, 1.0slot)</t>
         </is>
       </c>
       <c r="K6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>121949</v>
+        <v>112930</v>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Ferko, Lavdosh</t>
+          <t>Landis, Connor</t>
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D7" s="10" t="n">
         <v>32.5</v>
@@ -1565,61 +1565,61 @@
       </c>
       <c r="J7" s="13" t="inlineStr">
         <is>
-          <t>130 British Literature (English, 5.0cr, 1.0slot); 330 Spanish III (Language, 5.0cr, 1.0slot); 440 Precalculus (Mathematics, 5.0cr, 1.0slot); 530 Physics (Science, 5.0cr, 1.0slot); 631 CPR-AED Training/PE (Physical Education, 2.5cr, 0.5slot); 731 U.S. History II H (Social Studies, 5.0cr, 1.0slot); 830 Theology 11 (Theology, 5.0cr, 1.0slot)</t>
+          <t>120 American Literature (English, 5.0cr, 1.0slot); 322 Italian II (Language, 5.0cr, 1.0slot); 422 Geometry (Mathematics, 5.0cr, 1.0slot); 510 Biology (Science, 5.0cr, 1.0slot); 620 Driver's Ed/PE (Physical Education, 2.5cr, 0.5slot); 720 U.S. History I (Social Studies, 5.0cr, 1.0slot); 820 Theology 10 (Theology, 5.0cr, 1.0slot)</t>
         </is>
       </c>
       <c r="K7" s="9" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
-        <v>108187</v>
+        <v>109385</v>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Greig, Anthony</t>
+          <t>Saliba, Georges</t>
         </is>
       </c>
       <c r="C8" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D8" s="10" t="n">
-        <v>27.5</v>
+        <v>32.5</v>
       </c>
       <c r="E8" s="11" t="n">
-        <v>7.5</v>
+        <v>2.5</v>
       </c>
       <c r="F8" s="10" t="n">
-        <v>5.5</v>
+        <v>6.5</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I8" s="12" t="inlineStr">
         <is>
-          <t>Language</t>
+          <t>Physical Education</t>
         </is>
       </c>
       <c r="J8" s="13" t="inlineStr">
         <is>
-          <t>130 British Literature (English, 5.0cr, 1.0slot); 430 Algebra II/Trig (Mathematics, 5.0cr, 1.0slot); 530 Physics (Science, 5.0cr, 1.0slot); 631 CPR-AED Training/PE (Physical Education, 2.5cr, 0.5slot); 730 U.S. History II (Social Studies, 5.0cr, 1.0slot); 830 Theology 11 (Theology, 5.0cr, 1.0slot)</t>
+          <t>120 American Literature (English, 5.0cr, 1.0slot); 327 Latin II H (Language, 5.0cr, 1.0slot); 420 Geometry (Mathematics, 5.0cr, 1.0slot); 520 Chemistry (Science, 5.0cr, 1.0slot); 580 Robotics Engineering (Engineering, 2.5cr, 0.5slot); 720 U.S. History I (Social Studies, 5.0cr, 1.0slot); 820 Theology 10 (Theology, 5.0cr, 1.0slot)</t>
         </is>
       </c>
       <c r="K8" s="9" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
-        <v>112275</v>
+        <v>113831</v>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Kesselly, Brian</t>
+          <t>Sanchez, Cordero</t>
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D9" s="10" t="n">
         <v>32.5</v>
@@ -1643,96 +1643,96 @@
       </c>
       <c r="J9" s="13" t="inlineStr">
         <is>
-          <t>130 British Literature (English, 5.0cr, 1.0slot); 351 AP Spanish (Language, 5.0cr, 1.0slot); 450 Calculus H (Mathematics, 5.0cr, 1.0slot); 531 Physics H (Science, 5.0cr, 1.0slot); 580 Robotics Engineering (Engineering, 2.5cr, 0.5slot); 730 U.S. History II (Social Studies, 5.0cr, 1.0slot); 830 Theology 11 (Theology, 5.0cr, 1.0slot)</t>
+          <t>120 American Literature (English, 5.0cr, 1.0slot); 321 Spanish II H (Language, 5.0cr, 1.0slot); 421 Geometry H (Mathematics, 5.0cr, 1.0slot); 520 Chemistry (Science, 5.0cr, 1.0slot); 620 Driver's Ed/PE (Physical Education, 2.5cr, 0.5slot); 721 U.S. History I H (Social Studies, 5.0cr, 1.0slot); 820 Theology 10 (Theology, 5.0cr, 1.0slot)</t>
         </is>
       </c>
       <c r="K9" s="9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
-        <v>121320</v>
+        <v>121949</v>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Kirby, Benjamin</t>
+          <t>Ferko, Lavdosh</t>
         </is>
       </c>
       <c r="C10" s="5" t="n">
         <v>11</v>
       </c>
       <c r="D10" s="10" t="n">
-        <v>27.5</v>
+        <v>32.5</v>
       </c>
       <c r="E10" s="11" t="n">
-        <v>7.5</v>
+        <v>2.5</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>5.5</v>
+        <v>6.5</v>
       </c>
       <c r="G10" s="11" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I10" s="12" t="inlineStr">
         <is>
-          <t>Language</t>
+          <t>All core present — missing elective</t>
         </is>
       </c>
       <c r="J10" s="13" t="inlineStr">
         <is>
-          <t>130 British Literature (English, 5.0cr, 1.0slot); 443 AP Precalculus (Mathematics, 5.0cr, 1.0slot); 531 Physics H (Science, 5.0cr, 1.0slot); 631 CPR-AED Training/PE (Physical Education, 2.5cr, 0.5slot); 733 AP U.S. History (Social Studies, 5.0cr, 1.0slot); 830 Theology 11 (Theology, 5.0cr, 1.0slot)</t>
+          <t>130 British Literature (English, 5.0cr, 1.0slot); 330 Spanish III (Language, 5.0cr, 1.0slot); 440 Precalculus (Mathematics, 5.0cr, 1.0slot); 530 Physics (Science, 5.0cr, 1.0slot); 631 CPR-AED Training/PE (Physical Education, 2.5cr, 0.5slot); 731 U.S. History II H (Social Studies, 5.0cr, 1.0slot); 830 Theology 11 (Theology, 5.0cr, 1.0slot)</t>
         </is>
       </c>
       <c r="K10" s="9" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
-        <v>121986</v>
+        <v>108187</v>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Rodriguez, Blake</t>
+          <t>Greig, Anthony</t>
         </is>
       </c>
       <c r="C11" s="5" t="n">
         <v>11</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>32.5</v>
+        <v>27.5</v>
       </c>
       <c r="E11" s="11" t="n">
-        <v>2.5</v>
+        <v>7.5</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
       <c r="G11" s="11" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I11" s="12" t="inlineStr">
         <is>
-          <t>All core present — missing elective</t>
+          <t>Language</t>
         </is>
       </c>
       <c r="J11" s="13" t="inlineStr">
         <is>
-          <t>130 British Literature (English, 5.0cr, 1.0slot); 330 Spanish III (Language, 5.0cr, 1.0slot); 440 Precalculus (Mathematics, 5.0cr, 1.0slot); 530 Physics (Science, 5.0cr, 1.0slot); 631 CPR-AED Training/PE (Physical Education, 2.5cr, 0.5slot); 730 U.S. History II (Social Studies, 5.0cr, 1.0slot); 830 Theology 11 (Theology, 5.0cr, 1.0slot)</t>
+          <t>130 British Literature (English, 5.0cr, 1.0slot); 430 Algebra II/Trig (Mathematics, 5.0cr, 1.0slot); 530 Physics (Science, 5.0cr, 1.0slot); 631 CPR-AED Training/PE (Physical Education, 2.5cr, 0.5slot); 730 U.S. History II (Social Studies, 5.0cr, 1.0slot); 830 Theology 11 (Theology, 5.0cr, 1.0slot)</t>
         </is>
       </c>
       <c r="K11" s="9" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
-        <v>108153</v>
+        <v>112275</v>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Vagnone, Tyler</t>
+          <t>Kesselly, Brian</t>
         </is>
       </c>
       <c r="C12" s="5" t="n">
@@ -1760,61 +1760,61 @@
       </c>
       <c r="J12" s="13" t="inlineStr">
         <is>
-          <t>130 British Literature (English, 5.0cr, 1.0slot); 333 Italian III H (Language, 5.0cr, 1.0slot); 440 Precalculus (Mathematics, 5.0cr, 1.0slot); 531 Physics H (Science, 5.0cr, 1.0slot); 730 U.S. History II (Social Studies, 5.0cr, 1.0slot); 734 Leadership, Entrepreneurship and Opportunity Program I (Business, 2.5cr, 0.5slot); 830 Theology 11 (Theology, 5.0cr, 1.0slot)</t>
+          <t>130 British Literature (English, 5.0cr, 1.0slot); 351 AP Spanish (Language, 5.0cr, 1.0slot); 450 Calculus H (Mathematics, 5.0cr, 1.0slot); 531 Physics H (Science, 5.0cr, 1.0slot); 580 Robotics Engineering (Engineering, 2.5cr, 0.5slot); 730 U.S. History II (Social Studies, 5.0cr, 1.0slot); 830 Theology 11 (Theology, 5.0cr, 1.0slot)</t>
         </is>
       </c>
       <c r="K12" s="9" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
-        <v>106800</v>
+        <v>121320</v>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Wagner, Liran</t>
+          <t>Kirby, Benjamin</t>
         </is>
       </c>
       <c r="C13" s="5" t="n">
         <v>11</v>
       </c>
       <c r="D13" s="10" t="n">
-        <v>32.5</v>
+        <v>27.5</v>
       </c>
       <c r="E13" s="11" t="n">
-        <v>2.5</v>
+        <v>7.5</v>
       </c>
       <c r="F13" s="10" t="n">
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
       <c r="G13" s="11" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I13" s="12" t="inlineStr">
         <is>
-          <t>All core present — missing elective</t>
+          <t>Language</t>
         </is>
       </c>
       <c r="J13" s="13" t="inlineStr">
         <is>
-          <t>139 AP English Language (English, 5.0cr, 1.0slot); 331 Spanish III H (Language, 5.0cr, 1.0slot); 445 Adv Precalculus H (Mathematics, 5.0cr, 1.0slot); 557 AP Physics 1 (Science, 5.0cr, 1.0slot); 733 AP U.S. History (Social Studies, 5.0cr, 1.0slot); 734 Leadership, Entrepreneurship and Opportunity Program I (Business, 2.5cr, 0.5slot); 830 Theology 11 (Theology, 5.0cr, 1.0slot)</t>
+          <t>130 British Literature (English, 5.0cr, 1.0slot); 443 AP Precalculus (Mathematics, 5.0cr, 1.0slot); 531 Physics H (Science, 5.0cr, 1.0slot); 631 CPR-AED Training/PE (Physical Education, 2.5cr, 0.5slot); 733 AP U.S. History (Social Studies, 5.0cr, 1.0slot); 830 Theology 11 (Theology, 5.0cr, 1.0slot)</t>
         </is>
       </c>
       <c r="K13" s="9" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
-        <v>106291</v>
+        <v>119656</v>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Bonita, Andrew</t>
+          <t>Pierce, Dylan</t>
         </is>
       </c>
       <c r="C14" s="5" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D14" s="10" t="n">
         <v>32.5</v>
@@ -1829,7 +1829,7 @@
         <v>0.5</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I14" s="12" t="inlineStr">
         <is>
@@ -1838,22 +1838,22 @@
       </c>
       <c r="J14" s="13" t="inlineStr">
         <is>
-          <t>149 AP English Literature (English, 5.0cr, 1.0slot); 352 AP Italian (Language, 5.0cr, 1.0slot); 456 AP Statistics (Mathematics, 5.0cr, 1.0slot); 558 AP Physics C (Science, 5.0cr, 1.0slot); 642 Nutrition &amp; Fitness/PE (Physical Education, 2.5cr, 0.5slot); 765 AP Macroeconomics (Social Studies, 2.5cr, 0.5slot); 766 AP Microeconomics (Social Studies, 2.5cr, 0.5slot); 849 Catholic Social Teaching (Theology, 2.5cr, 0.5slot); 851 Spirituality of Vocation (Theology, 2.5cr, 0.5slot)</t>
+          <t>132 British Literature (English, 5.0cr, 1.0slot); 330 Spanish III (Language, 5.0cr, 1.0slot); 432 Algebra II/Trig (Mathematics, 5.0cr, 1.0slot); 530 Physics (Science, 5.0cr, 1.0slot); 720 U.S. History I (Social Studies, 5.0cr, 1.0slot); 727 Sports and Entertainment Marketing (Business, 2.5cr, 0.5slot); 830 Theology 11 (Theology, 5.0cr, 1.0slot)</t>
         </is>
       </c>
       <c r="K14" s="9" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
-        <v>107376</v>
+        <v>121986</v>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Carfello, Braydon</t>
+          <t>Rodriguez, Blake</t>
         </is>
       </c>
       <c r="C15" s="5" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D15" s="10" t="n">
         <v>32.5</v>
@@ -1868,7 +1868,7 @@
         <v>0.5</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="I15" s="12" t="inlineStr">
         <is>
@@ -1877,22 +1877,22 @@
       </c>
       <c r="J15" s="13" t="inlineStr">
         <is>
-          <t>140 World Literature (English, 5.0cr, 1.0slot); 242 Studio Art II (Art, 2.5cr, 0.5slot); 448 Pre-college Math (Mathematics, 5.0cr, 1.0slot); 546 Forensics (Science, 5.0cr, 1.0slot); 642 Nutrition &amp; Fitness/PE (Physical Education, 2.5cr, 0.5slot); 723 Introduction to Political Science (Social Studies, 2.5cr, 0.5slot); 741 Psychology (Social Studies, 2.5cr, 0.5slot); 751 American Government &amp; Politics (Social Studies, 2.5cr, 0.5slot); 849 Catholic Social Teaching (Theology, 2.5cr, 0.5slot); 851 Spirituality of Vocation (Theology, 2.5cr, 0.5slot)</t>
+          <t>130 British Literature (English, 5.0cr, 1.0slot); 330 Spanish III (Language, 5.0cr, 1.0slot); 440 Precalculus (Mathematics, 5.0cr, 1.0slot); 530 Physics (Science, 5.0cr, 1.0slot); 631 CPR-AED Training/PE (Physical Education, 2.5cr, 0.5slot); 730 U.S. History II (Social Studies, 5.0cr, 1.0slot); 830 Theology 11 (Theology, 5.0cr, 1.0slot)</t>
         </is>
       </c>
       <c r="K15" s="9" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
-        <v>106243</v>
+        <v>108153</v>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Duran, Nicholas</t>
+          <t>Vagnone, Tyler</t>
         </is>
       </c>
       <c r="C16" s="5" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D16" s="10" t="n">
         <v>32.5</v>
@@ -1907,7 +1907,7 @@
         <v>0.5</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="I16" s="12" t="inlineStr">
         <is>
@@ -1916,22 +1916,22 @@
       </c>
       <c r="J16" s="13" t="inlineStr">
         <is>
-          <t>141 College English Honors (English, 5.0cr, 1.0slot); 440 Precalculus (Mathematics, 5.0cr, 1.0slot); 544 Sports Medicine (Science, 5.0cr, 1.0slot); 595 Engineering Design (Engineering, 2.5cr, 0.5slot); 642 Nutrition &amp; Fitness/PE (Physical Education, 2.5cr, 0.5slot); 741 Psychology (Social Studies, 2.5cr, 0.5slot); 744 Sociology (Social Studies, 2.5cr, 0.5slot); 849 Catholic Social Teaching (Theology, 2.5cr, 0.5slot); 851 Spirituality of Vocation (Theology, 2.5cr, 0.5slot); 2044 TV/Film Production II (Communication Arts, 2.5cr, 0.5slot)</t>
+          <t>130 British Literature (English, 5.0cr, 1.0slot); 333 Italian III H (Language, 5.0cr, 1.0slot); 440 Precalculus (Mathematics, 5.0cr, 1.0slot); 531 Physics H (Science, 5.0cr, 1.0slot); 730 U.S. History II (Social Studies, 5.0cr, 1.0slot); 734 Leadership, Entrepreneurship and Opportunity Program I (Business, 2.5cr, 0.5slot); 830 Theology 11 (Theology, 5.0cr, 1.0slot)</t>
         </is>
       </c>
       <c r="K16" s="9" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
-        <v>106323</v>
+        <v>106800</v>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Gebert, Evan</t>
+          <t>Wagner, Liran</t>
         </is>
       </c>
       <c r="C17" s="5" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D17" s="10" t="n">
         <v>32.5</v>
@@ -1946,7 +1946,7 @@
         <v>0.5</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I17" s="12" t="inlineStr">
         <is>
@@ -1955,18 +1955,18 @@
       </c>
       <c r="J17" s="13" t="inlineStr">
         <is>
-          <t>141 College English Honors (English, 5.0cr, 1.0slot); 144 Public Speaking (English, 2.5cr, 0.5slot); 220 Music Theory (Music, 2.5cr, 0.5slot); 440 Precalculus (Mathematics, 5.0cr, 1.0slot); 546 Forensics (Science, 5.0cr, 1.0slot); 744 Sociology (Social Studies, 2.5cr, 0.5slot); 752 Economics H (Business, 5.0cr, 1.0slot); 849 Catholic Social Teaching (Theology, 2.5cr, 0.5slot); 851 Spirituality of Vocation (Theology, 2.5cr, 0.5slot)</t>
+          <t>139 AP English Language (English, 5.0cr, 1.0slot); 331 Spanish III H (Language, 5.0cr, 1.0slot); 445 Adv Precalculus H (Mathematics, 5.0cr, 1.0slot); 557 AP Physics 1 (Science, 5.0cr, 1.0slot); 733 AP U.S. History (Social Studies, 5.0cr, 1.0slot); 734 Leadership, Entrepreneurship and Opportunity Program I (Business, 2.5cr, 0.5slot); 830 Theology 11 (Theology, 5.0cr, 1.0slot)</t>
         </is>
       </c>
       <c r="K17" s="9" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
-        <v>112088</v>
+        <v>106291</v>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Helou, Ramsey</t>
+          <t>Bonita, Andrew</t>
         </is>
       </c>
       <c r="C18" s="5" t="n">
@@ -1985,7 +1985,7 @@
         <v>0.5</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I18" s="12" t="inlineStr">
         <is>
@@ -1994,37 +1994,37 @@
       </c>
       <c r="J18" s="13" t="inlineStr">
         <is>
-          <t>141 College English Honors (English, 5.0cr, 1.0slot); 144 Public Speaking (English, 2.5cr, 0.5slot); 145 Journalism (English, 2.5cr, 0.5slot); 450 Calculus H (Mathematics, 5.0cr, 1.0slot); 472 Web Design (Computer Science, 2.5cr, 0.5slot); 708 Introduction to Business (Business, 2.5cr, 0.5slot); 741 Psychology (Social Studies, 2.5cr, 0.5slot); 849 Catholic Social Teaching (Theology, 2.5cr, 0.5slot); 851 Spirituality of Vocation (Theology, 2.5cr, 0.5slot); 2044 TV/Film Production II (Communication Arts, 2.5cr, 0.5slot); 2054 Digital Media (Communication Arts, 2.5cr, 0.5slot)</t>
+          <t>149 AP English Literature (English, 5.0cr, 1.0slot); 352 AP Italian (Language, 5.0cr, 1.0slot); 456 AP Statistics (Mathematics, 5.0cr, 1.0slot); 558 AP Physics C (Science, 5.0cr, 1.0slot); 642 Nutrition &amp; Fitness/PE (Physical Education, 2.5cr, 0.5slot); 765 AP Macroeconomics (Social Studies, 2.5cr, 0.5slot); 766 AP Microeconomics (Social Studies, 2.5cr, 0.5slot); 849 Catholic Social Teaching (Theology, 2.5cr, 0.5slot); 851 Spirituality of Vocation (Theology, 2.5cr, 0.5slot)</t>
         </is>
       </c>
       <c r="K18" s="9" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
-        <v>106216</v>
+        <v>107376</v>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>McLaughlin, Sean</t>
+          <t>Carfello, Braydon</t>
         </is>
       </c>
       <c r="C19" s="5" t="n">
         <v>12</v>
       </c>
       <c r="D19" s="10" t="n">
-        <v>32.5</v>
+        <v>30</v>
       </c>
       <c r="E19" s="11" t="n">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="F19" s="10" t="n">
-        <v>6.5</v>
+        <v>6</v>
       </c>
       <c r="G19" s="11" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I19" s="12" t="inlineStr">
         <is>
@@ -2033,57 +2033,57 @@
       </c>
       <c r="J19" s="13" t="inlineStr">
         <is>
-          <t>141 College English Honors (English, 5.0cr, 1.0slot); 443 AP Precalculus (Mathematics, 5.0cr, 1.0slot); 557 AP Physics 1 (Science, 5.0cr, 1.0slot); 642 Nutrition &amp; Fitness/PE (Physical Education, 2.5cr, 0.5slot); 752 Economics H (Business, 5.0cr, 1.0slot); 757 International Business Strategies (Business, 5.0cr, 1.0slot); 849 Catholic Social Teaching (Theology, 2.5cr, 0.5slot); 851 Spirituality of Vocation (Theology, 2.5cr, 0.5slot)</t>
+          <t>140 World Literature (English, 5.0cr, 1.0slot); 242 Studio Art II (Art, 2.5cr, 0.5slot); 448 Pre-college Math (Mathematics, 5.0cr, 1.0slot); 546 Forensics (Science, 5.0cr, 1.0slot); 642 Nutrition &amp; Fitness/PE (Physical Education, 2.5cr, 0.5slot); 741 Psychology (Social Studies, 2.5cr, 0.5slot); 751 American Government &amp; Politics (Social Studies, 2.5cr, 0.5slot); 849 Catholic Social Teaching (Theology, 2.5cr, 0.5slot); 851 Spirituality of Vocation (Theology, 2.5cr, 0.5slot)</t>
         </is>
       </c>
       <c r="K19" s="9" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="n">
-        <v>106232</v>
+        <v>106243</v>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Nadler, Nathaniel</t>
+          <t>Duran, Nicholas</t>
         </is>
       </c>
       <c r="C20" s="5" t="n">
         <v>12</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>15</v>
+        <v>32.5</v>
       </c>
       <c r="E20" s="11" t="n">
-        <v>20</v>
+        <v>2.5</v>
       </c>
       <c r="F20" s="10" t="n">
-        <v>3</v>
+        <v>6.5</v>
       </c>
       <c r="G20" s="11" t="n">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="I20" s="12" t="inlineStr">
         <is>
-          <t>Mathematics</t>
+          <t>All core present — missing elective</t>
         </is>
       </c>
       <c r="J20" s="13" t="inlineStr">
         <is>
-          <t>149 AP English Literature (English, 5.0cr, 1.0slot); 763 AP U.S. Government &amp; Politics (Social Studies, 5.0cr, 1.0slot); 849 Catholic Social Teaching (Theology, 2.5cr, 0.5slot); 851 Spirituality of Vocation (Theology, 2.5cr, 0.5slot)</t>
+          <t>141 College English Honors (English, 5.0cr, 1.0slot); 440 Precalculus (Mathematics, 5.0cr, 1.0slot); 544 Sports Medicine (Science, 5.0cr, 1.0slot); 595 Engineering Design (Engineering, 2.5cr, 0.5slot); 642 Nutrition &amp; Fitness/PE (Physical Education, 2.5cr, 0.5slot); 741 Psychology (Social Studies, 2.5cr, 0.5slot); 744 Sociology (Social Studies, 2.5cr, 0.5slot); 849 Catholic Social Teaching (Theology, 2.5cr, 0.5slot); 851 Spirituality of Vocation (Theology, 2.5cr, 0.5slot); 2044 TV/Film Production II (Communication Arts, 2.5cr, 0.5slot)</t>
         </is>
       </c>
       <c r="K20" s="9" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n">
-        <v>106248</v>
+        <v>106323</v>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Strayton, Ryder</t>
+          <t>Gebert, Evan</t>
         </is>
       </c>
       <c r="C21" s="5" t="n">
@@ -2111,10 +2111,283 @@
       </c>
       <c r="J21" s="13" t="inlineStr">
         <is>
+          <t>141 College English Honors (English, 5.0cr, 1.0slot); 144 Public Speaking (English, 2.5cr, 0.5slot); 220 Music Theory (Music, 2.5cr, 0.5slot); 440 Precalculus (Mathematics, 5.0cr, 1.0slot); 546 Forensics (Science, 5.0cr, 1.0slot); 744 Sociology (Social Studies, 2.5cr, 0.5slot); 752 Economics H (Business, 5.0cr, 1.0slot); 849 Catholic Social Teaching (Theology, 2.5cr, 0.5slot); 851 Spirituality of Vocation (Theology, 2.5cr, 0.5slot)</t>
+        </is>
+      </c>
+      <c r="K21" s="9" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
+        <v>112088</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Helou, Ramsey</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D22" s="10" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="E22" s="11" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F22" s="10" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G22" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="I22" s="12" t="inlineStr">
+        <is>
+          <t>All core present — missing elective</t>
+        </is>
+      </c>
+      <c r="J22" s="13" t="inlineStr">
+        <is>
+          <t>141 College English Honors (English, 5.0cr, 1.0slot); 144 Public Speaking (English, 2.5cr, 0.5slot); 145 Journalism (English, 2.5cr, 0.5slot); 450 Calculus H (Mathematics, 5.0cr, 1.0slot); 472 Web Design (Computer Science, 2.5cr, 0.5slot); 708 Introduction to Business (Business, 2.5cr, 0.5slot); 741 Psychology (Social Studies, 2.5cr, 0.5slot); 849 Catholic Social Teaching (Theology, 2.5cr, 0.5slot); 851 Spirituality of Vocation (Theology, 2.5cr, 0.5slot); 2044 TV/Film Production II (Communication Arts, 2.5cr, 0.5slot); 2054 Digital Media (Communication Arts, 2.5cr, 0.5slot)</t>
+        </is>
+      </c>
+      <c r="K22" s="9" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
+        <v>106253</v>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>McLaughlin, Colin</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D23" s="10" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="E23" s="11" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F23" s="10" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G23" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="I23" s="12" t="inlineStr">
+        <is>
+          <t>All core present — missing elective</t>
+        </is>
+      </c>
+      <c r="J23" s="13" t="inlineStr">
+        <is>
+          <t>140 World Literature (English, 5.0cr, 1.0slot); 440 Precalculus (Mathematics, 5.0cr, 1.0slot); 546 Forensics (Science, 5.0cr, 1.0slot); 642 Nutrition &amp; Fitness/PE (Physical Education, 2.5cr, 0.5slot); 741 Psychology (Social Studies, 2.5cr, 0.5slot); 742 Economics (Business, 5.0cr, 1.0slot); 751 American Government &amp; Politics (Social Studies, 2.5cr, 0.5slot); 849 Catholic Social Teaching (Theology, 2.5cr, 0.5slot); 851 Spirituality of Vocation (Theology, 2.5cr, 0.5slot)</t>
+        </is>
+      </c>
+      <c r="K23" s="9" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="n">
+        <v>106216</v>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>McLaughlin, Sean</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D24" s="10" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="E24" s="11" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F24" s="10" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G24" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H24" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="I24" s="12" t="inlineStr">
+        <is>
+          <t>All core present — missing elective</t>
+        </is>
+      </c>
+      <c r="J24" s="13" t="inlineStr">
+        <is>
+          <t>141 College English Honors (English, 5.0cr, 1.0slot); 443 AP Precalculus (Mathematics, 5.0cr, 1.0slot); 557 AP Physics 1 (Science, 5.0cr, 1.0slot); 642 Nutrition &amp; Fitness/PE (Physical Education, 2.5cr, 0.5slot); 752 Economics H (Business, 5.0cr, 1.0slot); 757 International Business Strategies (Business, 5.0cr, 1.0slot); 849 Catholic Social Teaching (Theology, 2.5cr, 0.5slot); 851 Spirituality of Vocation (Theology, 2.5cr, 0.5slot)</t>
+        </is>
+      </c>
+      <c r="K24" s="9" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>106266</v>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Murphy, Finbar</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D25" s="10" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="E25" s="11" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F25" s="10" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G25" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="I25" s="12" t="inlineStr">
+        <is>
+          <t>All core present — missing elective</t>
+        </is>
+      </c>
+      <c r="J25" s="13" t="inlineStr">
+        <is>
+          <t>140 World Literature (English, 5.0cr, 1.0slot); 145 Journalism (English, 2.5cr, 0.5slot); 440 Precalculus (Mathematics, 5.0cr, 1.0slot); 472 Web Design (Computer Science, 2.5cr, 0.5slot); 544 Sports Medicine (Science, 5.0cr, 1.0slot); 642 Nutrition &amp; Fitness/PE (Physical Education, 2.5cr, 0.5slot); 849 Catholic Social Teaching (Theology, 2.5cr, 0.5slot); 851 Spirituality of Vocation (Theology, 2.5cr, 0.5slot); 2044 TV/Film Production II (Communication Arts, 2.5cr, 0.5slot); 2054 Digital Media (Communication Arts, 2.5cr, 0.5slot)</t>
+        </is>
+      </c>
+      <c r="K25" s="9" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n">
+        <v>106232</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Nadler, Nathaniel</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D26" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="E26" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="F26" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="G26" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H26" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I26" s="12" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="J26" s="13" t="inlineStr">
+        <is>
+          <t>149 AP English Literature (English, 5.0cr, 1.0slot); 763 AP U.S. Government &amp; Politics (Social Studies, 5.0cr, 1.0slot); 849 Catholic Social Teaching (Theology, 2.5cr, 0.5slot); 851 Spirituality of Vocation (Theology, 2.5cr, 0.5slot)</t>
+        </is>
+      </c>
+      <c r="K26" s="9" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n">
+        <v>106316</v>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Olivero Gamez, Josue</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D27" s="10" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="E27" s="11" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F27" s="10" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G27" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H27" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="I27" s="12" t="inlineStr">
+        <is>
+          <t>All core present — missing elective</t>
+        </is>
+      </c>
+      <c r="J27" s="13" t="inlineStr">
+        <is>
+          <t>140 World Literature (English, 5.0cr, 1.0slot); 351 AP Spanish (Language, 5.0cr, 1.0slot); 440 Precalculus (Mathematics, 5.0cr, 1.0slot); 546 Forensics (Science, 5.0cr, 1.0slot); 742 Economics (Business, 5.0cr, 1.0slot); 751 American Government &amp; Politics (Social Studies, 2.5cr, 0.5slot); 849 Catholic Social Teaching (Theology, 2.5cr, 0.5slot); 851 Spirituality of Vocation (Theology, 2.5cr, 0.5slot)</t>
+        </is>
+      </c>
+      <c r="K27" s="9" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="n">
+        <v>106248</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Strayton, Ryder</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D28" s="10" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="E28" s="11" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F28" s="10" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G28" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H28" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="I28" s="12" t="inlineStr">
+        <is>
+          <t>All core present — missing elective</t>
+        </is>
+      </c>
+      <c r="J28" s="13" t="inlineStr">
+        <is>
           <t>140 World Literature (English, 5.0cr, 1.0slot); 440 Precalculus (Mathematics, 5.0cr, 1.0slot); 546 Forensics (Science, 5.0cr, 1.0slot); 744 Sociology (Social Studies, 2.5cr, 0.5slot); 751 American Government &amp; Politics (Social Studies, 2.5cr, 0.5slot); 756 Introduction to Law (Social Studies, 2.5cr, 0.5slot); 761 AP Psychology (Social Studies, 5.0cr, 1.0slot); 849 Catholic Social Teaching (Theology, 2.5cr, 0.5slot); 851 Spirituality of Vocation (Theology, 2.5cr, 0.5slot)</t>
         </is>
       </c>
-      <c r="K21" s="9" t="inlineStr"/>
+      <c r="K28" s="9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>